<commit_message>
V2.3: Hierarquia de alertas (Grave primeiro) e correção de variável de data
</commit_message>
<xml_diff>
--- a/equipe/Alcides_Neto.xlsx
+++ b/equipe/Alcides_Neto.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SuporteLead\Desktop\dashboard_analytics\equipe\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SuporteLead\Desktop\dell-analytics-pro\equipe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E803E3D0-F5DE-4F59-93BB-7CB10B84E52F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BEB9722-6AFA-4068-B443-397126D63C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6756598C-5089-436D-B84C-2A58A92D56DF}"/>
   </bookViews>
@@ -734,7 +734,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N2" s="9">
         <v>0</v>

</xml_diff>